<commit_message>
Added getting achievement data
</commit_message>
<xml_diff>
--- a/Steam_Games.xlsx
+++ b/Steam_Games.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CJ\Documents\My Projects\My Skill Development\game-achievement-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ADEB1EC-BA1D-41D0-A6C9-4F2B13203FCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D253A60-2427-42FB-9280-25184DC0A834}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>ID</t>
   </si>
@@ -54,6 +54,9 @@
   </si>
   <si>
     <t>Black Myth Wukong</t>
+  </si>
+  <si>
+    <t>game_link</t>
   </si>
 </sst>
 </file>
@@ -95,7 +98,11 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -109,14 +116,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{507F0839-0555-426B-B7DB-068B4BAF2678}" name="Table1" displayName="Table1" ref="A1:C4" totalsRowShown="0">
-  <autoFilter ref="A1:C4" xr:uid="{507F0839-0555-426B-B7DB-068B4BAF2678}"/>
-  <tableColumns count="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{507F0839-0555-426B-B7DB-068B4BAF2678}" name="Table1" displayName="Table1" ref="A1:D4" totalsRowShown="0">
+  <autoFilter ref="A1:D4" xr:uid="{507F0839-0555-426B-B7DB-068B4BAF2678}"/>
+  <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{3E161485-89FB-41E6-A63E-4664D0B0ECB0}" name="ID">
       <calculatedColumnFormula>ROW()-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="2" xr3:uid="{007859EE-C1EE-44C6-BFAC-1E67740E87F2}" name="Game"/>
     <tableColumn id="3" xr3:uid="{C37BA298-9796-40A0-90DB-956803912E0C}" name="game_id"/>
+    <tableColumn id="4" xr3:uid="{A71223AC-FD24-4499-A224-DD876F6C628B}" name="game_link" dataDxfId="0">
+      <calculatedColumnFormula>"https://steamdb.info/app/"&amp;Table1[[#This Row],[game_id]]&amp;"/stats/"</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -385,10 +395,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -398,8 +408,11 @@
       <c r="C1" t="s">
         <v>4</v>
       </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
         <f>ROW()-1</f>
         <v>1</v>
@@ -410,8 +423,12 @@
       <c r="C2">
         <v>2358720</v>
       </c>
+      <c r="D2" t="str">
+        <f>"https://steamdb.info/app/"&amp;Table1[[#This Row],[game_id]]&amp;"/stats/"</f>
+        <v>https://steamdb.info/app/2358720/stats/</v>
+      </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3">
         <f>ROW()-1</f>
         <v>2</v>
@@ -422,8 +439,12 @@
       <c r="C3">
         <v>1627720</v>
       </c>
+      <c r="D3" t="str">
+        <f>"https://steamdb.info/app/"&amp;Table1[[#This Row],[game_id]]&amp;"/stats/"</f>
+        <v>https://steamdb.info/app/1627720/stats/</v>
+      </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4">
         <f>ROW()-1</f>
         <v>3</v>
@@ -433,6 +454,10 @@
       </c>
       <c r="C4">
         <v>1245620</v>
+      </c>
+      <c r="D4" t="str">
+        <f>"https://steamdb.info/app/"&amp;Table1[[#This Row],[game_id]]&amp;"/stats/"</f>
+        <v>https://steamdb.info/app/1245620/stats/</v>
       </c>
     </row>
   </sheetData>

</xml_diff>